<commit_message>
docs: review opensquilla for borrowable designs
</commit_message>
<xml_diff>
--- a/bench/devil-v25/AI-Agent_魔鬼训练_v2.5_AI独立评分表.xlsx
+++ b/bench/devil-v25/AI-Agent_魔鬼训练_v2.5_AI独立评分表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="13500"/>
+    <workbookView windowWidth="17280" windowHeight="26940"/>
   </bookViews>
   <sheets>
     <sheet name="AI-Agent_魔鬼训练_v2.5_AI独立评分表444" sheetId="1" r:id="rId1"/>
@@ -2913,9 +2913,10 @@
   <dimension ref="A1:I123"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="19.6666666666667" customWidth="1"/>
-    <col min="7" max="7" width="12.2222222222222" customWidth="1"/>
-    <col min="8" max="8" width="36.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="99" customWidth="1"/>
+    <col min="5" max="6" width="10" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="12.2222222222222" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="8.77777777777778" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">

</xml_diff>